<commit_message>
fix: align candidate import with updated template
</commit_message>
<xml_diff>
--- a/public/templates/Template_du_lieu_thi_sinh.xlsx
+++ b/public/templates/Template_du_lieu_thi_sinh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LAPTOP-NQ\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCB54CE-3790-49E6-8583-701292E3CAB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE51724-ED1E-400B-BE16-09E8A0066C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,10 +46,6 @@
     <t>Họ và tên thí sinh</t>
   </si>
   <si>
-    <t>Ngày sinh
-(DD/MM/YYYY hoặc YYYY)</t>
-  </si>
-  <si>
     <t>Số CCCD/Hộ chiếu</t>
   </si>
   <si>
@@ -59,26 +55,11 @@
     <t>Họ tên phụ huynh</t>
   </si>
   <si>
-    <t>Số điện thoại liên lạc</t>
-  </si>
-  <si>
-    <t>Email liên lạc</t>
-  </si>
-  <si>
-    <t>Tỉnh/Thành phố cư trú</t>
-  </si>
-  <si>
     <t>Địa chỉ liên hệ</t>
-  </si>
-  <si>
-    <t>Tên trường</t>
   </si>
   <si>
     <t>Lớp đang học
 (ví dụ: 6A1)</t>
-  </si>
-  <si>
-    <t>Khối lớp hiện tại</t>
   </si>
   <si>
     <t>Môn thi/Lĩnh vực</t>
@@ -94,9 +75,6 @@
   </si>
   <si>
     <t>Ngôn ngữ thi</t>
-  </si>
-  <si>
-    <t>Ghi chú chung</t>
   </si>
   <si>
     <t>Điều kiện tham gia</t>
@@ -160,6 +138,27 @@
   </si>
   <si>
     <t>Mật khẩu</t>
+  </si>
+  <si>
+    <t>Ngày sinh</t>
+  </si>
+  <si>
+    <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Tỉnh/Thành phố</t>
+  </si>
+  <si>
+    <t>Trường</t>
+  </si>
+  <si>
+    <t>Khối lớp</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
   </si>
 </sst>
 </file>
@@ -691,211 +690,211 @@
         <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="M2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="O2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="Q2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="2" t="s">
+      <c r="R2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="S2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="T2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="U2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="W2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="Y2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="Z2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="AA2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="AB2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AH2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AK2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="AL2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AN2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="AO2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="AP2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="AQ2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="AR2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AS2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AT2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AU2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AV2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AW2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="AX2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AY2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="AZ2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="BA2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="BB2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="BC2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="BD2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="BE2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="BF2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="BG2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="BH2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="BI2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="BJ2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="BK2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="BL2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="BM2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="BN2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="BO2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AD2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE2" s="4" t="s">
+      <c r="BP2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="BQ2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="BR2" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="AH2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ2" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="AL2" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="AM2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AN2" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AO2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="AP2" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AQ2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="AR2" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="AS2" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="AT2" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AU2" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="AV2" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AW2" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="AX2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="AY2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="AZ2" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="BA2" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="BB2" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="BC2" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="BD2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="BE2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="BF2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="BG2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="BH2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="BI2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="BJ2" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="BK2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="BL2" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="BM2" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="BN2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="BO2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="BP2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="BQ2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="BR2" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:70" ht="17.55" customHeight="1">

</xml_diff>